<commit_message>
record tile destinations and recount the tiles
All 46 tile destinations opened 14 September 2026. Every one
resolves; none redirects. Results added to the listings workbook
as destination page and destination note, and to
documents/tile-link-check.tsv.

The Biostatistics and Foundational Mathematics tiles are down,
taking the count from 48 to 46 and closing two of the
catalog-against-tiles discrepancies. Mathematics, Single Subject
Matter Preparation moves to the no-tile list.

The graduate program directory page now returns 404, leaving the
Program Coordinator link on the prospective graduate students
page dead. Divya Sitaraman's email is corrected on the Graduate
Studies page; the facilitator title is not.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/graduate-program-listings.xlsx
+++ b/committee/grad-facilitator/documents/graduate-program-listings.xlsx
@@ -537,7 +537,7 @@
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Compiled 10 September 2026 by I. Thiebaut.</t>
+          <t>Compiled 10 September 2026 by I. Thiebaut. Tile destinations opened and tiles recounted 14 September 2026.</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Whether the program has a tile. "unresolved" marks Mathematics, Single Subject Matter Preparation, where the tiles carry Mathematics, Single Subject Matter and Foundational Mathematics, Single Subject and which names which is an open question.</t>
+          <t>Whether the program has a tile on the Office of Graduate Studies page.</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>/graduate-studies/graduate-program-directory.html is tagged “Unused page. Do not publish.” and is live. The prospective graduate students page sends applicants there for program coordinator contacts. It carries no Music tile and links into catalog years 33 and 39.</t>
+          <t>/graduate-studies/graduate-program-directory.html returns 404 as of 14 September 2026. The prospective graduate students page still sends applicants to it for program coordinator contacts, under Departmental Admission Requirements, so that link is now dead. The Important Links block on the same page points to graduate-program-coordinators.html, which resolves.</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Divya Sitaraman’s email is listed as joshua.kerr@csueastbay.edu. The graduate recruitment facilitator is listed as a Graduate Student Success Facilitator.</t>
+          <t>Divya Sitaraman’s email is corrected as of 14 September 2026. The graduate recruitment facilitator is still listed as a Graduate Student Success Facilitator.</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The tile links have not been opened, except Accountancy, which reaches the MS in Accountancy program page.</t>
+          <t>All 46 tiles were opened on 14 September 2026. Every one resolves. The destination page and destination note columns carry what each one reaches. Fourteen tiles share six URLs. The Educational Technology certificate is the only tile pointing into the catalog rather than a program page, and it points into catalog year 39.</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,8 @@
     <col width="46" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -816,6 +818,16 @@
           <t>note</t>
         </is>
       </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>destination page</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>destination note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -863,6 +875,12 @@
           <t>self-support only, delivered through university extension, placed here provisionally, department to confirm</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Post-Baccalaureate Health Professions Academic Program</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -906,6 +924,12 @@
           <t>tracks: with PASC, with optional PASC</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Masters in Educational Leadership</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -949,6 +973,12 @@
           <t>summer admission</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Doctorate in Educational Leadership for Social Justice</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -992,6 +1022,12 @@
           <t>available self-support</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Preliminary Administrative Services Credential (PASC) /Optional Masters in Educational Leadership</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -1035,6 +1071,12 @@
           <t>not in the catalog</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Administrative Services Clear Induction Program</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1082,6 +1124,12 @@
           <t>concentrations: Marriage and Family Therapy, School Counseling, School Psychology</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Graduate Programs</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1121,6 +1169,12 @@
       </c>
       <c r="H8" s="8" t="inlineStr"/>
       <c r="I8" s="8" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>School Counseling</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1160,6 +1214,12 @@
       </c>
       <c r="H9" s="8" t="inlineStr"/>
       <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Prospective Students &amp; Application Process</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1203,6 +1263,16 @@
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Master's Degree</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1246,6 +1316,16 @@
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Master's Degree</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1289,6 +1369,16 @@
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Master's Degree</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1332,6 +1422,12 @@
           <t>self-support only</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Reading and Literacy</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1375,6 +1471,12 @@
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Multiple Subject Credential Program</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1418,6 +1520,12 @@
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Single Subject Credential Program</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1461,6 +1569,16 @@
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>(page carries no title)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>points into catalog year 39; returned no content to an automated request</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1508,6 +1626,16 @@
           <t>concentrations: Extensive Support Needs, Mild/Moderate Support Needs</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Education Specialist/Masters in Special Education - Online Program</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1551,6 +1679,16 @@
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Education Specialist/Masters in Special Education - Online Program</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1594,6 +1732,16 @@
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>IxDIA, Master of Arts in Interaction Design and Interactive Art</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>off the university domain</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1672,6 +1820,12 @@
       </c>
       <c r="H21" s="8" t="inlineStr"/>
       <c r="I21" s="8" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>(page carries no title)</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1750,6 +1904,12 @@
       </c>
       <c r="H23" s="8" t="inlineStr"/>
       <c r="I23" s="8" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>M.S. in Hospitality, Recreation and Tourism</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1789,6 +1949,12 @@
       </c>
       <c r="H24" s="8" t="inlineStr"/>
       <c r="I24" s="8" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>M.A. in Music</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1828,6 +1994,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr"/>
       <c r="I25" s="8" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Music Education</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1867,6 +2039,12 @@
       </c>
       <c r="H26" s="8" t="inlineStr"/>
       <c r="I26" s="8" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Master's of Science Health Care Administration Program</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1910,6 +2088,12 @@
           <t>concentrations: Health Care Administration, Public Management and Policy Analysis</t>
         </is>
       </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Master's Degree in Public Administration</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1949,6 +2133,12 @@
       </c>
       <c r="H28" s="8" t="inlineStr"/>
       <c r="I28" s="8" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>GRADUATE PROGRAMS</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1992,6 +2182,12 @@
           <t>administered by Moss Landing Marine Laboratories</t>
         </is>
       </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>MS in Marine Sciences</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2031,6 +2227,12 @@
       </c>
       <c r="H30" s="8" t="inlineStr"/>
       <c r="I30" s="8" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Prospective and Current BCP Students</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -2074,6 +2276,12 @@
           <t>concentrations: Chemistry, Biochemistry</t>
         </is>
       </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Master of Science in Chemistry</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -2117,6 +2325,12 @@
           <t>concentrations: Artificial Intelligence and Machine Learning, Computer Networks, Computer Science</t>
         </is>
       </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Computer Science Degrees</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -2156,6 +2370,12 @@
       </c>
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -2199,6 +2419,16 @@
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>GRADUATE DEGREES</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -2242,6 +2472,16 @@
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>GRADUATE DEGREES</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2285,6 +2525,16 @@
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>CSUEB Math Degrees and Programs</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2328,6 +2578,16 @@
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>CSUEB Math Degrees and Programs</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -2352,7 +2612,7 @@
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
@@ -2363,7 +2623,7 @@
       <c r="G38" s="9" t="inlineStr"/>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>the tiles carry Mathematics, Single Subject Matter and Foundational Mathematics, Single Subject; which of the two catalog entries each names is an open question</t>
+          <t>the one Math single subject matter tile is named Mathematics, Single Subject Matter and matches the certificate</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr"/>
@@ -2391,18 +2651,14 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr"/>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>https://www.csueastbay.edu/math/degrees-and-programs/index.html</t>
-        </is>
-      </c>
+      <c r="G39" s="13" t="n"/>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>tile only; shared with Mathematics, M.S. and the Mathematics Single Subject Matter tile</t>
+          <t>tile removed on or before 14 September 2026</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -2410,6 +2666,8 @@
           <t>not in the catalog under this name; the Mathematics degrees and programs page lists no foundational-level program</t>
         </is>
       </c>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -2457,6 +2715,16 @@
           <t>concentrations: Actuarial Science, Applied Statistics, Biostatistics, Data Science, Mathematical Statistics</t>
         </is>
       </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Programs in Statistics and Data Science</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -2500,6 +2768,16 @@
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Programs in Statistics and Data Science</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -2543,6 +2821,16 @@
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Programs in Statistics and Data Science</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 3 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -2567,18 +2855,14 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F43" s="12" t="inlineStr"/>
-      <c r="G43" s="13" t="inlineStr">
-        <is>
-          <t>https://www.csueastbay.edu/statistics/biostatistics-psm/index.html</t>
-        </is>
-      </c>
+      <c r="G43" s="13" t="n"/>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>tile only</t>
+          <t>tile removed on or before 14 September 2026</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
@@ -2633,6 +2917,12 @@
           <t>self-support only</t>
         </is>
       </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Master of Science in Accountancy</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -2711,6 +3001,12 @@
       </c>
       <c r="H46" s="8" t="inlineStr"/>
       <c r="I46" s="8" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Master of Science in Business Analytics- College of Business &amp; Economics | CSUEB</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -2750,6 +3046,12 @@
       </c>
       <c r="H47" s="8" t="inlineStr"/>
       <c r="I47" s="8" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Master of Science in Marketing Analytics- College of Business &amp; Economics | CSUEB</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -2793,6 +3095,12 @@
           <t>concentrations delivered across departments: Finance, General Business, General Business One-Year Accelerated (self-support), Human Resources Management and Organizational Behavior, Marketing Management, Operations and Supply Chain Management</t>
         </is>
       </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Master of Business Administration- College of Business and Economics | CSUEB</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -2836,6 +3144,12 @@
           <t>concentrations: Human Movement and Sport Science, Physical Activity and Exercise</t>
         </is>
       </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>M.S. Kinesiology: Sport, exercise, and human movement</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -2914,6 +3228,12 @@
       </c>
       <c r="H51" s="8" t="inlineStr"/>
       <c r="I51" s="8" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>MSN Program</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -2957,6 +3277,12 @@
           <t>tracks: standard, advanced standing</t>
         </is>
       </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Apply to the MSW Program</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -3000,6 +3326,16 @@
         </is>
       </c>
       <c r="I53" s="8" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Master's in Speech-Language Pathology</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -3043,6 +3379,16 @@
         </is>
       </c>
       <c r="I54" s="8" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Master's in Speech-Language Pathology</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>url shared by 2 tiles</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I54"/>
@@ -3117,34 +3463,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
record shared tile destinations as department pages
A destination serving several tiles is the department page for
those programs, not a link fault. Reworded in programs.md, in the
destination note column, and in the read me tab.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/graduate-program-listings.xlsx
+++ b/committee/grad-facilitator/documents/graduate-program-listings.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>All 46 tiles were opened on 14 September 2026. Every one resolves. The destination page and destination note columns carry what each one reaches. Fourteen tiles share six URLs. The Educational Technology certificate is the only tile pointing into the catalog rather than a program page, and it points into catalog year 39.</t>
+          <t>All 46 tiles were opened on 14 September 2026. Every one resolves. The destination page and destination note columns carry what each one reaches. Six destinations serve more than one tile, each the department page holding those programs. The Educational Technology certificate is the only tile pointing into the catalog rather than a program page, and it points into catalog year 39.</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>url shared by 3 tiles</t>
+          <t>department page for 3 of the tiles</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>url shared by 2 tiles</t>
+          <t>department page for 2 of the tiles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
move shared destinations into the note column
A destination serving several tiles is recorded as a fact about
the program rather than as a link issue, in both the roster tables
and the listings workbook. The Foundational Mathematics tile is
out of the Mathematics rows.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/graduate-program-listings.xlsx
+++ b/committee/grad-facilitator/documents/graduate-program-listings.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>What the Graduate Studies tile does that needs a look: a shared link, a different name, an archived catalog year. Blank means nothing noted.</t>
+          <t>What the Graduate Studies tile does that needs a look: a different name, an archived catalog year. Blank means nothing noted. A destination shared by several tiles is recorded in the note column.</t>
         </is>
       </c>
     </row>
@@ -1257,12 +1257,12 @@
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>shared with Early Childhood Education and Educational Technology</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Early Childhood Education and Educational Technology</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Master's Degree</t>
@@ -1310,12 +1310,12 @@
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>shared with Curriculum and Instruction and Educational Technology</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Curriculum and Instruction and Educational Technology</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Master's Degree</t>
@@ -1363,12 +1363,12 @@
           <t>https://www.csueastbay.edu/ted/programs-admissions/masters/index.html</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>shared with Curriculum and Instruction and Early Childhood Education</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Curriculum and Instruction and Early Childhood Education</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Master's Degree</t>
@@ -1616,14 +1616,10 @@
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/special-education.html</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>shared with the Education Specialist Credential</t>
-        </is>
-      </c>
+      <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>concentrations: Extensive Support Needs, Mild/Moderate Support Needs</t>
+          <t>concentrations: Extensive Support Needs, Mild/Moderate Support Needs; department page shared with the Education Specialist Credential</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1673,12 +1669,12 @@
           <t>https://www.csueastbay.edu/cssc/prospective-cred-student/special-education.html</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>shared with Special Education, M.S.</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Special Education, M.S.</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Education Specialist/Masters in Special Education - Online Program</t>
@@ -2413,12 +2409,12 @@
           <t>https://www.csueastbay.edu/engineering/programs-degrees/graduate-degrees.html</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>shared with Engineering Management</t>
-        </is>
-      </c>
-      <c r="I34" s="8" t="inlineStr"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Engineering Management</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
           <t>GRADUATE DEGREES</t>
@@ -2466,12 +2462,12 @@
           <t>https://www.csueastbay.edu/engineering/programs-degrees/graduate-degrees.html</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
-        <is>
-          <t>shared with Construction Management</t>
-        </is>
-      </c>
-      <c r="I35" s="8" t="inlineStr"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Construction Management</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
           <t>GRADUATE DEGREES</t>
@@ -2519,12 +2515,12 @@
           <t>https://www.csueastbay.edu/math/degrees-and-programs/index.html</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>shared with the Foundational Mathematics and Mathematics Single Subject Matter tiles</t>
-        </is>
-      </c>
-      <c r="I36" s="8" t="inlineStr"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with the Mathematics Single Subject Matter certificate</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
           <t>CSUEB Math Degrees and Programs</t>
@@ -2574,10 +2570,14 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>tile is named Mathematics, Single Subject Matter; shared with Mathematics, M.S. and the Foundational Mathematics tile</t>
-        </is>
-      </c>
-      <c r="I37" s="8" t="inlineStr"/>
+          <t>tile is named Mathematics, Single Subject Matter</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Mathematics, M.S.</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
           <t>CSUEB Math Degrees and Programs</t>
@@ -2705,14 +2705,10 @@
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>shared with the Applied Statistics and Theoretical Statistics tiles</t>
-        </is>
-      </c>
+      <c r="H40" s="8" t="n"/>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>concentrations: Actuarial Science, Applied Statistics, Biostatistics, Data Science, Mathematical Statistics</t>
+          <t>concentrations: Actuarial Science, Applied Statistics, Biostatistics, Data Science, Mathematical Statistics; department page shared with the Applied Statistics and Theoretical Statistics certificates</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2762,12 +2758,12 @@
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>shared with Statistics, M.S. and the Theoretical Statistics tile</t>
-        </is>
-      </c>
-      <c r="I41" s="8" t="inlineStr"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Statistics, M.S. and the Theoretical Statistics certificate</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Programs in Statistics and Data Science</t>
@@ -2815,12 +2811,12 @@
           <t>https://www.csueastbay.edu/statistics/degrees-programs/index.html</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>shared with Statistics, M.S. and the Applied Statistics tile</t>
-        </is>
-      </c>
-      <c r="I42" s="8" t="inlineStr"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Statistics, M.S. and the Applied Statistics certificate</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Programs in Statistics and Data Science</t>
@@ -3320,12 +3316,12 @@
           <t>https://www.csueastbay.edu/slhs/masters-in-speech-language-pathology/index.html</t>
         </is>
       </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>shared with the Speech Language Pathology Services credential tile</t>
-        </is>
-      </c>
-      <c r="I53" s="8" t="inlineStr"/>
+      <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with the Speech Language Pathology Services credential</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Master's in Speech-Language Pathology</t>
@@ -3373,12 +3369,12 @@
           <t>https://www.csueastbay.edu/slhs/masters-in-speech-language-pathology/index.html</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
-        <is>
-          <t>shared with Speech-Language Pathology, M.S.</t>
-        </is>
-      </c>
-      <c r="I54" s="8" t="inlineStr"/>
+      <c r="H54" s="8" t="n"/>
+      <c r="I54" s="8" t="inlineStr">
+        <is>
+          <t>department page shared with Speech-Language Pathology, M.S.</t>
+        </is>
+      </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Master's in Speech-Language Pathology</t>

</xml_diff>